<commit_message>
Deploy TWHA IG: 4 項送審前覆核決議 (LDL/FVC/anti-HCV/腰圍) — tx 0 Error
對應原始碼 commit 427dbbc。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/StructureDefinition-TWHA-PulmonaryFunction.xlsx
+++ b/StructureDefinition-TWHA-PulmonaryFunction.xlsx
@@ -63,7 +63,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-25T16:18:15+08:00</t>
+    <t>2026-07-26T10:07:44+08:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -697,8 +697,8 @@
     <t>&lt;valueCodeableConcept xmlns="http://hl7.org/fhir"&gt;
   &lt;coding&gt;
     &lt;system value="http://loinc.org"/&gt;
-    &lt;code value="19876-2"/&gt;
-    &lt;display value="Forced vital capacity [Volume] Respiratory system by Spirometry --pre bronchodilation"/&gt;
+    &lt;code value="19868-9"/&gt;
+    &lt;display value="Forced vital capacity [Volume] Respiratory system by Spirometry"/&gt;
   &lt;/coding&gt;
 &lt;/valueCodeableConcept&gt;</t>
   </si>

</xml_diff>